<commit_message>
feat(sync): otomatis salin master_user_pic.xlsx ke folder Downloads dan perjelas panduan upload ke Google Drive
</commit_message>
<xml_diff>
--- a/data/master_user_pic.xlsx
+++ b/data/master_user_pic.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:J13"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -796,9 +796,41 @@
         <v>2026-10-30T10:01:36.672Z</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="str">
+        <v>105515</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Chandra</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Teknik</v>
+      </c>
+      <c r="E13" t="str">
+        <v>IT</v>
+      </c>
+      <c r="F13" t="str">
+        <v>super_admin</v>
+      </c>
+      <c r="G13" t="str">
+        <v>R99</v>
+      </c>
+      <c r="H13" t="str">
+        <v>105515@pelindo.co.id</v>
+      </c>
+      <c r="I13" t="str">
+        <v>AKTIF</v>
+      </c>
+      <c r="J13" t="str">
+        <v>2026-10-30T10:09:33.189Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J13"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -848,7 +880,7 @@
         <v>Terakhir Disinkronkan</v>
       </c>
       <c r="B5" t="str">
-        <v>2026-10-30T10:08:19.811Z</v>
+        <v>2026-10-30T10:15:34.030Z</v>
       </c>
     </row>
     <row r="6">
@@ -856,7 +888,7 @@
         <v>Total PIC Terdaftar</v>
       </c>
       <c r="B6">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: tambahkan menu data per periode dan input data manual semua modul
</commit_message>
<xml_diff>
--- a/data/master_user_pic.xlsx
+++ b/data/master_user_pic.xlsx
@@ -452,7 +452,7 @@
         <v>10000</v>
       </c>
       <c r="C2" t="str">
-        <v>Board of Directors (BOD)</v>
+        <v>Akhirman (BOD)</v>
       </c>
       <c r="D2" t="str">
         <v>Direksi Pelindo Regional 4</v>
@@ -484,7 +484,7 @@
         <v>10001</v>
       </c>
       <c r="C3" t="str">
-        <v>Budi Santoso, S.T., M.M.</v>
+        <v>M Mansyur</v>
       </c>
       <c r="D3" t="str">
         <v>Divisi Teknologi Informasi &amp; Digitalisasi</v>
@@ -516,7 +516,7 @@
         <v>10002</v>
       </c>
       <c r="C4" t="str">
-        <v>Hendra Wijaya, S.E., M.B.A.</v>
+        <v>Asqar</v>
       </c>
       <c r="D4" t="str">
         <v>Divisi Strategi &amp; Manajemen Kinerja Regional</v>
@@ -548,7 +548,7 @@
         <v>10003</v>
       </c>
       <c r="C5" t="str">
-        <v>Capt. Rudi Hartono, M.Mar.</v>
+        <v>Heiruddin</v>
       </c>
       <c r="D5" t="str">
         <v>Divisi Operasi &amp; Pelayanan Kapal</v>
@@ -580,7 +580,7 @@
         <v>10004</v>
       </c>
       <c r="C6" t="str">
-        <v>Ahmad Dahlan, S.T.</v>
+        <v>Nuka</v>
       </c>
       <c r="D6" t="str">
         <v>Divisi Operasional Terminal Cabang</v>
@@ -612,7 +612,7 @@
         <v>10005</v>
       </c>
       <c r="C7" t="str">
-        <v>Siti Rahma, S.E., Ak., CA.</v>
+        <v>Rahmat Syukur</v>
       </c>
       <c r="D7" t="str">
         <v>Divisi Keuangan &amp; Manajemen Risiko</v>
@@ -644,7 +644,7 @@
         <v>10006</v>
       </c>
       <c r="C8" t="str">
-        <v>Dewi Kartika, S.Psi., M.M.</v>
+        <v>Arkam</v>
       </c>
       <c r="D8" t="str">
         <v>Divisi Sumber Daya Manusia &amp; Umum</v>
@@ -676,7 +676,7 @@
         <v>10007</v>
       </c>
       <c r="C9" t="str">
-        <v>Ir. Agus Santoso, M.T.</v>
+        <v>Abri</v>
       </c>
       <c r="D9" t="str">
         <v>Divisi Fasilitas &amp; Peralatan Pelabuhan</v>
@@ -708,7 +708,7 @@
         <v>10008</v>
       </c>
       <c r="C10" t="str">
-        <v>Faisal Ramadhan, S.Tr.Pel.</v>
+        <v>Fachruddin</v>
       </c>
       <c r="D10" t="str">
         <v>Divisi Operasional Terminal Cabang</v>
@@ -740,7 +740,7 @@
         <v>10009</v>
       </c>
       <c r="C11" t="str">
-        <v>Nur Aini, S.Kom.</v>
+        <v>Angga</v>
       </c>
       <c r="D11" t="str">
         <v>Divisi Operasional Terminal Cabang</v>
@@ -772,7 +772,7 @@
         <v>10020</v>
       </c>
       <c r="C12" t="str">
-        <v>Bambang Sudiro, S.T.</v>
+        <v>Cakra Aulia</v>
       </c>
       <c r="D12" t="str">
         <v>Divisi Operasional Terminal</v>
@@ -880,7 +880,7 @@
         <v>Terakhir Disinkronkan</v>
       </c>
       <c r="B5" t="str">
-        <v>2026-11-01T01:19:20.829Z</v>
+        <v>2026-11-01T01:55:33.127Z</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
feat(auth): sesuaikan konfigurasi dashboard dan kunci cabang otomatis untuk role PIC Cabang
</commit_message>
<xml_diff>
--- a/data/master_user_pic.xlsx
+++ b/data/master_user_pic.xlsx
@@ -33,8 +33,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
+  <numFmts count="4">
+    <numFmt numFmtId="41" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
+    <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;_);_(@_)"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -880,7 +883,7 @@
         <v>Terakhir Disinkronkan</v>
       </c>
       <c r="B5" t="str">
-        <v>2026-11-01T01:55:33.127Z</v>
+        <v>2026-11-01T03:21:41.113Z</v>
       </c>
     </row>
     <row r="6">

</xml_diff>